<commit_message>
To Be Continue ..
+ Quest 정보
</commit_message>
<xml_diff>
--- a/Assets/02Script/Table/EventTable.xlsx
+++ b/Assets/02Script/Table/EventTable.xlsx
@@ -7,6 +7,7 @@
     <sheet state="visible" name="Narration" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="Dialog" sheetId="3" r:id="rId6"/>
     <sheet state="visible" name="Choice" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="Quest" sheetId="5" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -14,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1147" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1271" uniqueCount="421">
   <si>
     <t>EventID</t>
   </si>
@@ -910,8 +911,7 @@
     <t>E041</t>
   </si>
   <si>
-    <t>밖에 나가기엔 늦은 시간이야..
-내일을 위해서 어서 자야 해.</t>
+    <t>열쇠를 다 찾기 전까진 돌아갈 수 없어..</t>
   </si>
   <si>
     <t>Choice0</t>
@@ -1121,6 +1121,193 @@
   </si>
   <si>
     <t>N011</t>
+  </si>
+  <si>
+    <t>C011</t>
+  </si>
+  <si>
+    <t>지금은 분명 가을인데..</t>
+  </si>
+  <si>
+    <t>봄이었던 것 같기도 하고..?
+기억이 잘 안 나네..</t>
+  </si>
+  <si>
+    <t>N014_0</t>
+  </si>
+  <si>
+    <t>N014_1</t>
+  </si>
+  <si>
+    <t>N014</t>
+  </si>
+  <si>
+    <t>QuestID</t>
+  </si>
+  <si>
+    <t>ActiveID</t>
+  </si>
+  <si>
+    <t>DeactiveID</t>
+  </si>
+  <si>
+    <t>Q001</t>
+  </si>
+  <si>
+    <t>공원 출구 찾기.</t>
+  </si>
+  <si>
+    <t>Q002</t>
+  </si>
+  <si>
+    <t>위쪽 샛길 확인하기.</t>
+  </si>
+  <si>
+    <t>Q003</t>
+  </si>
+  <si>
+    <t>N003</t>
+  </si>
+  <si>
+    <t>시루와 대화하기.</t>
+  </si>
+  <si>
+    <t>Q004</t>
+  </si>
+  <si>
+    <t>샛길 밖으로 이동하기.</t>
+  </si>
+  <si>
+    <t>Q005</t>
+  </si>
+  <si>
+    <t>Q006</t>
+  </si>
+  <si>
+    <t>Q007</t>
+  </si>
+  <si>
+    <t>풍선 확인하기.</t>
+  </si>
+  <si>
+    <t>Q008</t>
+  </si>
+  <si>
+    <t>Q009</t>
+  </si>
+  <si>
+    <t>N005</t>
+  </si>
+  <si>
+    <t>문 확인하기.</t>
+  </si>
+  <si>
+    <t>Q010</t>
+  </si>
+  <si>
+    <t>공원 한가운데 수상한 공간 확인하기.</t>
+  </si>
+  <si>
+    <t>Q011</t>
+  </si>
+  <si>
+    <t>무성해 보이는 숲길 확인하기.</t>
+  </si>
+  <si>
+    <t>Q012</t>
+  </si>
+  <si>
+    <t>미로를 탐험하며 열쇠 찾기( N / 3).</t>
+  </si>
+  <si>
+    <t>Q013</t>
+  </si>
+  <si>
+    <t>귀신을 피해 탈출하기.</t>
+  </si>
+  <si>
+    <t>Q014</t>
+  </si>
+  <si>
+    <t>열쇠를 사용해 문 열기.</t>
+  </si>
+  <si>
+    <t>Q015</t>
+  </si>
+  <si>
+    <t>교실을 나가 집으로 돌아가기.</t>
+  </si>
+  <si>
+    <t>Q016</t>
+  </si>
+  <si>
+    <t>N012</t>
+  </si>
+  <si>
+    <t>침대로 가서 잠자기.</t>
+  </si>
+  <si>
+    <t>Q017</t>
+  </si>
+  <si>
+    <t>집으로 가는 길 찾기.</t>
+  </si>
+  <si>
+    <t>Q018</t>
+  </si>
+  <si>
+    <t>골목 안 확인하기.</t>
+  </si>
+  <si>
+    <t>Q019</t>
+  </si>
+  <si>
+    <t>양아치와 대화하기.</t>
+  </si>
+  <si>
+    <t>Q020</t>
+  </si>
+  <si>
+    <t>골목 밖으로 나가기.</t>
+  </si>
+  <si>
+    <t>Q021</t>
+  </si>
+  <si>
+    <t>Q022</t>
+  </si>
+  <si>
+    <t>소리가 들리는 곳 확인하기.</t>
+  </si>
+  <si>
+    <t>Q023</t>
+  </si>
+  <si>
+    <t>Q024</t>
+  </si>
+  <si>
+    <t>Q025</t>
+  </si>
+  <si>
+    <t>Q026</t>
+  </si>
+  <si>
+    <t>Q027</t>
+  </si>
+  <si>
+    <t>N013</t>
+  </si>
+  <si>
+    <t>Q028</t>
+  </si>
+  <si>
+    <t>도로 한가운데 수상한 공간 확인하기.</t>
+  </si>
+  <si>
+    <t>Q029</t>
+  </si>
+  <si>
+    <t>터널 안쪽 확인하기.</t>
   </si>
 </sst>
 </file>
@@ -1196,7 +1383,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1351,6 +1538,9 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1421,6 +1611,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="C2:C14" displayName="Table_1" name="Table_1" id="1">
   <tableColumns count="1">
@@ -1461,7 +1655,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="D81:J150" displayName="Table_4" name="Table_4" id="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="D81:J152" displayName="Table_4" name="Table_4" id="4">
   <tableColumns count="7">
     <tableColumn name="Column1" id="1"/>
     <tableColumn name="Column2" id="2"/>
@@ -6994,10 +7188,10 @@
       <c r="E150" s="41">
         <v>-1.0</v>
       </c>
-      <c r="F150" s="42" t="s">
-        <v>133</v>
-      </c>
-      <c r="G150" s="42" t="s">
+      <c r="F150" s="36" t="s">
+        <v>133</v>
+      </c>
+      <c r="G150" s="36" t="s">
         <v>134</v>
       </c>
       <c r="H150" s="36"/>
@@ -7011,10 +7205,24 @@
     <row r="151">
       <c r="A151" s="44"/>
       <c r="B151" s="44"/>
+      <c r="D151" s="42"/>
+      <c r="E151" s="18"/>
+      <c r="F151" s="36"/>
+      <c r="G151" s="36"/>
+      <c r="H151" s="36"/>
+      <c r="I151" s="38"/>
+      <c r="J151" s="28"/>
     </row>
     <row r="152">
       <c r="A152" s="44"/>
       <c r="B152" s="44"/>
+      <c r="D152" s="42"/>
+      <c r="E152" s="18"/>
+      <c r="F152" s="36"/>
+      <c r="G152" s="36"/>
+      <c r="H152" s="36"/>
+      <c r="I152" s="38"/>
+      <c r="J152" s="28"/>
     </row>
     <row r="153">
       <c r="A153" s="44"/>
@@ -10327,10 +10535,6 @@
     <row r="980">
       <c r="A980" s="44"/>
       <c r="B980" s="44"/>
-    </row>
-    <row r="981">
-      <c r="A981" s="44"/>
-      <c r="B981" s="44"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -10652,6 +10856,464 @@
         <v>358</v>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>359</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>360</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>361</v>
+      </c>
+      <c r="E12" s="3">
+        <v>-10.0</v>
+      </c>
+      <c r="F12" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>362</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>364</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="13.88"/>
+    <col customWidth="1" min="3" max="3" width="15.5"/>
+    <col customWidth="1" min="4" max="4" width="26.5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="s">
+        <v>365</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>366</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>367</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>368</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" s="52" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>370</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="49" t="s">
+        <v>30</v>
+      </c>
+      <c r="D3" s="52" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="49" t="s">
+        <v>373</v>
+      </c>
+      <c r="D4" s="52" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>373</v>
+      </c>
+      <c r="C5" s="49" t="s">
+        <v>36</v>
+      </c>
+      <c r="D5" s="52" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="49" t="s">
+        <v>42</v>
+      </c>
+      <c r="D6" s="52" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="s">
+        <v>378</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="D7" s="52" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="49" t="s">
+        <v>322</v>
+      </c>
+      <c r="D8" s="52" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>322</v>
+      </c>
+      <c r="C9" s="49" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="52" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="49" t="s">
+        <v>383</v>
+      </c>
+      <c r="D10" s="52" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="C11" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="52" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="s">
+        <v>387</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="49" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="52" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="49" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="52" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="s">
+        <v>391</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C14" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="52" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="s">
+        <v>393</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="52"/>
+      <c r="D15" s="52" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="s">
+        <v>395</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="49" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="52" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="s">
+        <v>397</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="49" t="s">
+        <v>398</v>
+      </c>
+      <c r="D17" s="52" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="s">
+        <v>400</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C18" s="49" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="52" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="49" t="s">
+        <v>80</v>
+      </c>
+      <c r="D19" s="52" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C20" s="49" t="s">
+        <v>352</v>
+      </c>
+      <c r="D20" s="52" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="C21" s="49" t="s">
+        <v>86</v>
+      </c>
+      <c r="D21" s="52" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C22" s="49" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="52" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C23" s="49" t="s">
+        <v>92</v>
+      </c>
+      <c r="D23" s="52" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C24" s="49" t="s">
+        <v>94</v>
+      </c>
+      <c r="D24" s="52" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>358</v>
+      </c>
+      <c r="C25" s="49" t="s">
+        <v>358</v>
+      </c>
+      <c r="D25" s="52" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="C26" s="49" t="s">
+        <v>98</v>
+      </c>
+      <c r="D26" s="52" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" s="49" t="s">
+        <v>100</v>
+      </c>
+      <c r="D27" s="52" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="C28" s="49" t="s">
+        <v>416</v>
+      </c>
+      <c r="D28" s="52" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="C29" s="49" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" s="52" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D30" s="52" t="s">
+        <v>420</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>